<commit_message>
data(referencia): atualiza governador do Espirito Santo apos sucessao
Renato Casagrande renunciou ao governo do ES em 2026-04-02 para
disputar o Senado; o vice Ricardo Ferraco assumiu definitivamente o
cargo na mesma data (fonte: planejamento.es.gov.br, confirmado pelo
usuario). Atualiza a linha do ES em governadores.xlsx:

- Governador: Renato Casagrande -> Ricardo Ferraco
- Partido: PSB -> MDB
- Vice-governador(a): Ricardo Ferraco -> Camillo Neves (confirmado
  pelo usuario)

Mandato (2019-2027) e Eleicao (2018, 2022) mantidos sem alteracao --
continuam descrevendo o mandato/chapa original, nao quem ocupa o cargo
hoje; nao alterados por falta de confirmacao sobre a semantica
pretendida desses campos apos uma sucessao.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/governadores.xlsx
+++ b/reference/governadores.xlsx
@@ -784,12 +784,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Renato Casagrande </t>
+          <t>Ricardo Ferraço</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PSB </t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Ricardo Ferraço </t>
+          <t>Camillo Neves</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">

</xml_diff>